<commit_message>
Remove unused supplementary figures. Add weighted continental mean to the dataset.
</commit_message>
<xml_diff>
--- a/Supplementary Data 1 - Metadata and Codebook.xlsx
+++ b/Supplementary Data 1 - Metadata and Codebook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kschne34\Dropbox\GitHub\FSCI2025_Performance_Replication\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ACAACCE-F5E4-4BF9-AC4A-E53333F6258B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A39DCD5-99DD-442F-9DE0-A91275112CDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" tabRatio="758" xr2:uid="{627FC470-C124-47B7-9254-ED9E29476D78}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" tabRatio="758" activeTab="2" xr2:uid="{627FC470-C124-47B7-9254-ED9E29476D78}"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="30" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4725" uniqueCount="1179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4727" uniqueCount="1179">
   <si>
     <t>Food Systems Countdown Initiative</t>
   </si>
@@ -4319,7 +4319,7 @@
       </c>
       <c r="B4" s="6">
         <f ca="1">TODAY()</f>
-        <v>46121</v>
+        <v>46122</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -9614,7 +9614,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
         <v>373</v>
       </c>
@@ -9635,7 +9635,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="8" t="s">
         <v>376</v>
       </c>
@@ -9656,7 +9656,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
         <v>379</v>
       </c>
@@ -9677,7 +9677,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="84" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>407</v>
       </c>
@@ -9698,7 +9698,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="85" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>431</v>
       </c>
@@ -9719,7 +9719,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>435</v>
       </c>
@@ -9740,7 +9740,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>439</v>
       </c>
@@ -9760,8 +9760,14 @@
       <c r="G87" s="8" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H87" s="8" t="s">
+        <v>416</v>
+      </c>
+      <c r="I87">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>539</v>
       </c>
@@ -9781,8 +9787,14 @@
       <c r="G88" s="8" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H88" s="8" t="s">
+        <v>416</v>
+      </c>
+      <c r="I88">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="1"/>
       <c r="B89" s="1"/>
       <c r="C89" s="7"/>
@@ -9790,7 +9802,7 @@
       <c r="E89" s="1"/>
       <c r="F89" s="1"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="1"/>
       <c r="B90" s="1"/>
       <c r="C90" s="7"/>
@@ -9798,7 +9810,7 @@
       <c r="E90" s="1"/>
       <c r="F90" s="1"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="1"/>
       <c r="B91" s="1"/>
       <c r="C91" s="7"/>
@@ -9806,7 +9818,7 @@
       <c r="E91" s="1"/>
       <c r="F91" s="1"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="1"/>
       <c r="B92" s="1"/>
       <c r="C92" s="7"/>
@@ -9814,7 +9826,7 @@
       <c r="E92" s="1"/>
       <c r="F92" s="1"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="1"/>
       <c r="B93" s="1"/>
       <c r="C93" s="7"/>
@@ -9822,7 +9834,7 @@
       <c r="E93" s="1"/>
       <c r="F93" s="1"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="1"/>
       <c r="B94" s="1"/>
       <c r="C94" s="7"/>
@@ -9830,12 +9842,12 @@
       <c r="E94" s="1"/>
       <c r="F94" s="1"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="1"/>
       <c r="B95" s="1"/>
       <c r="C95" s="7"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="1"/>
       <c r="B96" s="1"/>
       <c r="C96" s="7"/>
@@ -48711,21 +48723,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010018141AFBEDAA4E4F8F497BA0BA465628" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="51632a301ac108a956373b15242a2c1c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="3740b2bf-318f-4c2d-92fe-b8cc5ab95724" xmlns:ns4="0d38da4c-d0a5-4e53-81d3-71f1e08ba0ee" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8aed9f36c2f7cc18b5698afd23e33de4" ns3:_="" ns4:_="">
     <xsd:import namespace="3740b2bf-318f-4c2d-92fe-b8cc5ab95724"/>
@@ -48954,24 +48951,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2FF79C2-D6CA-4146-8A33-8B2F68A6926A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8B78A5C-B87B-48A6-A425-F525FA87B0A7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{629B1C7C-1368-414C-B746-5D693F4D5577}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -48988,4 +48983,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8B78A5C-B87B-48A6-A425-F525FA87B0A7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2FF79C2-D6CA-4146-8A33-8B2F68A6926A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>